<commit_message>
CI Reports [2026-06-25 18:29]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/DailyBugReport_2026-06-25.xlsx
+++ b/Test Execution Report/Daily Reports/DailyBugReport_2026-06-25.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:O16"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -708,9 +708,499 @@
         <v/>
       </c>
     </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>BUG-ALL-006</v>
+      </c>
+      <c r="C7" t="str">
+        <v>All</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TC-TICKET-005</v>
+      </c>
+      <c r="E7" t="str">
+        <v>[FAIL] TC-TICKET-005 | All Ticket Type chips are visible</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G7" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H7" t="str">
+        <v>New</v>
+      </c>
+      <c r="I7" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J7" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L7" t="str">
+        <v xml:space="preserve">Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('text=SCR').first() Expected: visible Received: hidden Timeout:  5000ms  Call log: _x001b_[2m  - </v>
+      </c>
+      <c r="M7" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N7" t="str">
+        <v>reports/screenshots/TC-TICKET-005-failure.png</v>
+      </c>
+      <c r="O7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>BUG-ALL-007</v>
+      </c>
+      <c r="C8" t="str">
+        <v>All</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TC-TICKET-006</v>
+      </c>
+      <c r="E8" t="str">
+        <v>[FAIL] TC-TICKET-006 | Description character counter updates on input</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G8" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H8" t="str">
+        <v>New</v>
+      </c>
+      <c r="I8" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J8" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mnot_x001b_[2m._x001b_[22mtoBe_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m) // Object.is equality_x001b_[22m  Expected: not _x001b_[32m"0 / 2000"_x001b_[39m</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N8" t="str">
+        <v>reports/screenshots/TC-TICKET-006-failure.png</v>
+      </c>
+      <c r="O8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>BUG-ALL-008</v>
+      </c>
+      <c r="C9" t="str">
+        <v>All</v>
+      </c>
+      <c r="D9" t="str">
+        <v>TC-TICKET-007</v>
+      </c>
+      <c r="E9" t="str">
+        <v>[FAIL] TC-TICKET-007 | Reset button clears all filled fields</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G9" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H9" t="str">
+        <v>New</v>
+      </c>
+      <c r="I9" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J9" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBe_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m) // Object.is equality_x001b_[22m  Expected: _x001b_[32m""_x001b_[39m Received: _x001b_[31m"Some description text here"_x001b_[39m</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N9" t="str">
+        <v>reports/screenshots/TC-TICKET-007-failure.png</v>
+      </c>
+      <c r="O9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>BUG-ALL-009</v>
+      </c>
+      <c r="C10" t="str">
+        <v>All</v>
+      </c>
+      <c r="D10" t="str">
+        <v>TC-TICKET-014</v>
+      </c>
+      <c r="E10" t="str">
+        <v>[FAIL] TC-TICKET-014 | Description with exactly 14 chars fails validation</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G10" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H10" t="str">
+        <v>New</v>
+      </c>
+      <c r="I10" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J10" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L10" t="str">
+        <v xml:space="preserve">Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoMatch_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m)_x001b_[22m  Expected pattern: _x001b_[32m/Description/i_x001b_[39m Received string:  _x001b_[31m"Are you sure you want to log this </v>
+      </c>
+      <c r="M10" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N10" t="str">
+        <v>reports/screenshots/TC-TICKET-014-failure.png</v>
+      </c>
+      <c r="O10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>BUG-ALL-010</v>
+      </c>
+      <c r="C11" t="str">
+        <v>All</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TC-TICKET-016</v>
+      </c>
+      <c r="E11" t="str">
+        <v>[FAIL] TC-TICKET-016 | Description at 2000 chars (max) is accepted</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G11" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H11" t="str">
+        <v>New</v>
+      </c>
+      <c r="I11" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J11" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBe_x001b_[2m(_x001b_[22m_x001b_[32mexpected_x001b_[39m_x001b_[2m) // Object.is equality_x001b_[22m  Expected: _x001b_[32m2000_x001b_[39m Received: _x001b_[31m0_x001b_[39m</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N11" t="str">
+        <v>reports/screenshots/TC-TICKET-016-failure.png</v>
+      </c>
+      <c r="O11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>BUG-ALL-011</v>
+      </c>
+      <c r="C12" t="str">
+        <v>All</v>
+      </c>
+      <c r="D12" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="E12" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G12" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H12" t="str">
+        <v>New</v>
+      </c>
+      <c r="I12" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J12" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M12" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N12" t="str">
+        <v>reports/screenshots/TC-DASH-002-failure.png</v>
+      </c>
+      <c r="O12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13" xml:space="preserve">
+      <c r="A13" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>BUG-ALL-012</v>
+      </c>
+      <c r="C13" t="str">
+        <v>All</v>
+      </c>
+      <c r="D13" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="E13" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G13" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H13" t="str">
+        <v>New</v>
+      </c>
+      <c r="I13" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J13" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M13" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N13" t="str">
+        <v>reports/screenshots/TC-DASH-004-failure.png</v>
+      </c>
+      <c r="O13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14" xml:space="preserve">
+      <c r="A14" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>BUG-ALL-013</v>
+      </c>
+      <c r="C14" t="str">
+        <v>All</v>
+      </c>
+      <c r="D14" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="E14" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G14" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H14" t="str">
+        <v>New</v>
+      </c>
+      <c r="I14" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J14" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M14" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N14" t="str">
+        <v>reports/screenshots/TC-DASH-005-failure.png</v>
+      </c>
+      <c r="O14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15" xml:space="preserve">
+      <c r="A15" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>BUG-ALL-014</v>
+      </c>
+      <c r="C15" t="str">
+        <v>All</v>
+      </c>
+      <c r="D15" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="E15" t="str">
+        <v>[FAIL] TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G15" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H15" t="str">
+        <v>New</v>
+      </c>
+      <c r="I15" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J15" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('button:has-text("Reset")').first() Expected: visible Received: hidden Timeout:  5000ms  Ca</v>
+      </c>
+      <c r="M15" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N15" t="str">
+        <v>reports/screenshots/TC-DASH-007-failure.png</v>
+      </c>
+      <c r="O15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16" xml:space="preserve">
+      <c r="A16" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>BUG-ALL-015</v>
+      </c>
+      <c r="C16" t="str">
+        <v>All</v>
+      </c>
+      <c r="D16" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="E16" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G16" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H16" t="str">
+        <v>New</v>
+      </c>
+      <c r="I16" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J16" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
+      </c>
+      <c r="M16" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N16" t="str">
+        <v>reports/screenshots/TC-DASH-011-failure.png</v>
+      </c>
+      <c r="O16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-06-25 19:15]: All — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report/Daily Reports/DailyBugReport_2026-06-25.xlsx
+++ b/Test Execution Report/Daily Reports/DailyBugReport_2026-06-25.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O21"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -1198,9 +1198,254 @@
         <v/>
       </c>
     </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>BUG-ALL-016</v>
+      </c>
+      <c r="C17" t="str">
+        <v>All</v>
+      </c>
+      <c r="D17" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="E17" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G17" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H17" t="str">
+        <v>New</v>
+      </c>
+      <c r="I17" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M17" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N17" t="str">
+        <v>reports/screenshots/TC-DASH-002-failure.png</v>
+      </c>
+      <c r="O17" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>BUG-ALL-017</v>
+      </c>
+      <c r="C18" t="str">
+        <v>All</v>
+      </c>
+      <c r="D18" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="E18" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G18" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H18" t="str">
+        <v>New</v>
+      </c>
+      <c r="I18" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M18" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N18" t="str">
+        <v>reports/screenshots/TC-DASH-004-failure.png</v>
+      </c>
+      <c r="O18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>BUG-ALL-018</v>
+      </c>
+      <c r="C19" t="str">
+        <v>All</v>
+      </c>
+      <c r="D19" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="E19" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G19" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H19" t="str">
+        <v>New</v>
+      </c>
+      <c r="I19" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mreceived_x001b_[39m_x001b_[2m)._x001b_[22mtoBeTruthy_x001b_[2m()_x001b_[22m  Received: _x001b_[31mfalse_x001b_[39m</v>
+      </c>
+      <c r="M19" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N19" t="str">
+        <v>reports/screenshots/TC-DASH-005-failure.png</v>
+      </c>
+      <c r="O19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>BUG-ALL-019</v>
+      </c>
+      <c r="C20" t="str">
+        <v>All</v>
+      </c>
+      <c r="D20" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="E20" t="str">
+        <v>[FAIL] TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G20" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H20" t="str">
+        <v>New</v>
+      </c>
+      <c r="I20" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('button:has-text("Reset")').first() Expected: visible Received: hidden Timeout:  5000ms  Ca</v>
+      </c>
+      <c r="M20" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N20" t="str">
+        <v>reports/screenshots/TC-DASH-007-failure.png</v>
+      </c>
+      <c r="O20" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>25 Jun 2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>BUG-ALL-020</v>
+      </c>
+      <c r="C21" t="str">
+        <v>All</v>
+      </c>
+      <c r="D21" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="E21" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G21" t="str">
+        <v>P3</v>
+      </c>
+      <c r="H21" t="str">
+        <v>New</v>
+      </c>
+      <c r="I21" t="str">
+        <v>http://customerportal.dev-ts.online | Chrome | Ubuntu</v>
+      </c>
+      <c r="J21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Navigate
+2. Execute test
+3. Observe failure</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Test should pass</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Error: _x001b_[2mexpect(_x001b_[22m_x001b_[31mlocator_x001b_[39m_x001b_[2m)._x001b_[22mtoBeVisible_x001b_[2m(_x001b_[22m_x001b_[2m)_x001b_[22m failed  Locator:  locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout:  5000ms  Cal</v>
+      </c>
+      <c r="M21" t="str">
+        <v>Automation (Playwright)</v>
+      </c>
+      <c r="N21" t="str">
+        <v>reports/screenshots/TC-DASH-011-failure.png</v>
+      </c>
+      <c r="O21" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>